<commit_message>
Update V-SMART Pro system
</commit_message>
<xml_diff>
--- a/รายชื่อพนักงานขับรถยนต์.xlsx
+++ b/รายชื่อพนักงานขับรถยนต์.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\v-smart\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33E4D394-AFD1-4B8D-8B35-DE4F7CF1044E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{01734D14-F796-40EF-A114-104A05CF7438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A69A46FB-0B2C-4AB7-922E-D85394636A8B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="48">
   <si>
     <t>ลำดับ</t>
   </si>
@@ -147,13 +147,49 @@
   </si>
   <si>
     <t>ข้อมูลรายชื่อผู้ใช้งานระบบ V-Smart</t>
+  </si>
+  <si>
+    <t>นายสืบศักดิ์ วงศ์สิงห์แก้ว</t>
+  </si>
+  <si>
+    <t>นายภูริภัทร ชัยยะเลิศ</t>
+  </si>
+  <si>
+    <t>น.ส.วรรณภา กันทะ</t>
+  </si>
+  <si>
+    <t>น.ส.นุศรา ปัญญาเหล็ก</t>
+  </si>
+  <si>
+    <t>นายสุวัชญ์ศิษฏ์ พุทธเดชากุล</t>
+  </si>
+  <si>
+    <t>นายสุชาติ อินยะ</t>
+  </si>
+  <si>
+    <t>กองสวัสดิการสังคม</t>
+  </si>
+  <si>
+    <t>ผู้ช่วยเจ้าพนักงานธุรการ</t>
+  </si>
+  <si>
+    <t>นักวิชาการการเงินและบัญชี</t>
+  </si>
+  <si>
+    <t>นักพัฒนาชุมชน</t>
+  </si>
+  <si>
+    <t>นิติกร</t>
+  </si>
+  <si>
+    <t>ไม่มีข้อมูล</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -171,13 +207,6 @@
     <font>
       <sz val="16"/>
       <color theme="1"/>
-      <name val="TH Sarabun New"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="16"/>
-      <color rgb="FF1F1F1F"/>
       <name val="TH Sarabun New"/>
       <family val="2"/>
     </font>
@@ -224,20 +253,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -245,9 +265,19 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -583,282 +613,376 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30329A67-676C-4AA6-B1C5-3347D7178C74}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="22.05" customHeight="1" x14ac:dyDescent="0.7"/>
   <cols>
-    <col min="1" max="1" width="7.19921875" style="3" customWidth="1"/>
-    <col min="2" max="2" width="7.796875" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.09765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.19921875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="7.796875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.296875" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.3984375" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25.19921875" style="1" customWidth="1"/>
     <col min="6" max="16384" width="8.796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="8" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:5" s="5" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A1" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
     </row>
     <row r="2" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A2" s="2"/>
+      <c r="A2" s="9"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A4" s="4">
+      <c r="A4" s="3">
         <v>1</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="3">
         <v>1234</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A5" s="4">
+      <c r="A5" s="3">
         <v>2</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="3">
         <v>2026</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A6" s="4">
+      <c r="A6" s="3">
         <v>3</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="3">
         <v>3456</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A7" s="4">
+      <c r="A7" s="3">
         <v>4</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="3">
         <v>4321</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A8" s="4">
+      <c r="A8" s="3">
         <v>5</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="3">
         <v>5678</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A9" s="4">
+      <c r="A9" s="3">
         <v>6</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="3">
         <v>6789</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A10" s="4">
+      <c r="A10" s="3">
         <v>7</v>
       </c>
-      <c r="B10" s="6">
+      <c r="B10" s="3">
         <v>7890</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A11" s="4">
+      <c r="A11" s="3">
         <v>8</v>
       </c>
-      <c r="B11" s="6">
+      <c r="B11" s="3">
         <v>8123</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A12" s="4">
+      <c r="A12" s="3">
         <v>9</v>
       </c>
-      <c r="B12" s="6">
+      <c r="B12" s="3">
         <v>9012</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A13" s="4">
+      <c r="A13" s="3">
         <v>10</v>
       </c>
-      <c r="B13" s="6">
+      <c r="B13" s="3">
         <v>1073</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A14" s="4">
+      <c r="A14" s="3">
         <v>11</v>
       </c>
-      <c r="B14" s="6">
+      <c r="B14" s="3">
         <v>1122</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="4" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A15" s="4">
+      <c r="A15" s="3">
         <v>12</v>
       </c>
-      <c r="B15" s="6">
+      <c r="B15" s="3">
         <v>8801</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="4" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A16" s="4">
+      <c r="A16" s="3">
         <v>13</v>
       </c>
-      <c r="B16" s="6">
+      <c r="B16" s="3">
         <v>1357</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="4" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A17" s="4">
+      <c r="A17" s="3">
         <v>14</v>
       </c>
-      <c r="B17" s="6">
+      <c r="B17" s="3">
         <v>1468</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="4" t="s">
         <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A18" s="6">
+        <v>15</v>
+      </c>
+      <c r="B18" s="6"/>
+      <c r="C18" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A19" s="6">
+        <v>16</v>
+      </c>
+      <c r="B19" s="6"/>
+      <c r="C19" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A20" s="6">
+        <v>17</v>
+      </c>
+      <c r="B20" s="6"/>
+      <c r="C20" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A21" s="6">
+        <v>18</v>
+      </c>
+      <c r="B21" s="6"/>
+      <c r="C21" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A22" s="6">
+        <v>19</v>
+      </c>
+      <c r="B22" s="6"/>
+      <c r="C22" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A23" s="6">
+        <v>20</v>
+      </c>
+      <c r="B23" s="6"/>
+      <c r="C23" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>